<commit_message>
alter template to display all data
</commit_message>
<xml_diff>
--- a/app/server/static/templates/reports/Dairy_Client_Details_Template.xlsx
+++ b/app/server/static/templates/reports/Dairy_Client_Details_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\MALS\app\server\static\templates\reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikeg\Desktop\work\nr-mals\app\server\static\templates\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96ACE093-CB7E-42D5-82E6-13BEBEC43F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3293F11F-B23C-4271-A691-F7424C761B70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{11309506-049F-4A42-8D72-2555D662D497}"/>
+    <workbookView xWindow="-28920" yWindow="5280" windowWidth="29040" windowHeight="15840" xr2:uid="{11309506-049F-4A42-8D72-2555D662D497}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Threshold Report" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="130">
   <si>
     <t>IH</t>
   </si>
@@ -231,13 +231,205 @@
   </si>
   <si>
     <t>Site Status:</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].IRMA_NUM}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Status}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].LicenceHolderCompany}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].LastnameFirstName}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Phone}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Address}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Fax}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].City} {d.Client[i+1].Province}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Cell}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Postcode}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Email}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].IssueDate}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].SiteStatus}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].SiteAddress}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].SiteCity} {d.Client[i+1].SiteProvince}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].TankCompany}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].TankModel}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].TankSerial}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].TankCapacity}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].LastInspectionDate}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].LastInspector}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Insp[i].Date}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Insp[i].IH}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Insp[i].SCC}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Insp[i].IBC}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Insp[i].CRY}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Insp[i+1].Date}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Avg_IH}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Avg_SCC}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Avg_IBC}</t>
+  </si>
+  <si>
+    <t>{d.Client[i+1].Avg_CRY}</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(IRMA:) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(City / Province) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Site Address:) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Site Status:) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Date) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Report Average) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(IH) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(0.15) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Contact:) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Client:) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Site) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Details) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Make) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Model) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Serial #) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Capacity) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(SCC) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(IBC) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(CRY) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(400000) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(121000) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(3.7) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Last Inspected On:) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Last Inspected By:) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Email:) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Cell:) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Fax:) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Phone:) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Postcode) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Address) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Name) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Status:) }</t>
+  </si>
+  <si>
+    <t>{ d.Client[i+1]:ifNEM():show(Issue Date:) }</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -261,6 +453,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -282,7 +480,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -305,20 +503,13 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -327,52 +518,39 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -687,7 +865,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6B4FD09-964A-4163-B64E-5BD98D9AE9F8}">
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
@@ -700,31 +878,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="F1" s="33" t="s">
+      <c r="B1" s="5"/>
+      <c r="F1" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
       <c r="J1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B3" s="2"/>
@@ -742,7 +920,7 @@
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="17" t="s">
         <v>63</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -751,59 +929,59 @@
       <c r="D5" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
     </row>
     <row r="7" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="17" t="s">
         <v>34</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="13"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" t="s">
         <v>35</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -812,13 +990,13 @@
       <c r="D10" t="s">
         <v>42</v>
       </c>
-      <c r="E10" s="13"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="19" t="s">
         <v>27</v>
       </c>
       <c r="B11" t="s">
@@ -830,13 +1008,13 @@
       <c r="D11" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="13"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="25" t="s">
+      <c r="A12" s="19" t="s">
         <v>28</v>
       </c>
       <c r="B12" t="s">
@@ -848,13 +1026,13 @@
       <c r="D12" t="s">
         <v>44</v>
       </c>
-      <c r="E12" s="13"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="19" t="s">
         <v>29</v>
       </c>
       <c r="B13" t="s">
@@ -866,45 +1044,45 @@
       <c r="D13" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="13"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="11" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="35" t="s">
+      <c r="A16" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="11" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="25" t="s">
+      <c r="A17" s="19" t="s">
         <v>14</v>
       </c>
       <c r="B17" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D17" s="2" t="s">
@@ -921,13 +1099,13 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="25" t="s">
+      <c r="A18" s="19" t="s">
         <v>28</v>
       </c>
       <c r="B18" t="s">
         <v>41</v>
       </c>
-      <c r="C18" s="27" t="s">
+      <c r="C18" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D18" t="s">
@@ -944,28 +1122,24 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="25"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
+      <c r="A19" s="19"/>
+      <c r="C19" s="14"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="16"/>
-      <c r="B20" s="15"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
+      <c r="A20" s="13"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="14"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="20" t="s">
+      <c r="A21" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="20" t="s">
+      <c r="C21" s="16" t="s">
         <v>15</v>
       </c>
       <c r="D21" t="s">
@@ -991,66 +1165,59 @@
       <c r="A24" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="21">
+      <c r="B24" s="7">
         <v>0.15</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="5">
         <v>400000</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="5">
         <v>121000</v>
       </c>
-      <c r="E24" s="21">
+      <c r="E24" s="7">
         <v>3.7</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="31" t="s">
+      <c r="A25" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="B25" s="31" t="s">
+      <c r="B25" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C25" s="31" t="s">
+      <c r="C25" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="D25" s="31" t="s">
+      <c r="D25" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="E25" s="31" t="s">
+      <c r="E25" s="10" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="31" t="s">
+      <c r="A26" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B26" s="28"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="29"/>
+      <c r="B26" s="21"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="29"/>
-      <c r="B27" s="28"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
+      <c r="B27" s="21"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="30" t="s">
+      <c r="A28" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="B28" s="32" t="s">
+      <c r="B28" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="32" t="s">
+      <c r="C28" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="D28" s="32" t="s">
+      <c r="D28" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E28" s="32" t="s">
+      <c r="E28" s="23" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1059,13 +1226,308 @@
       <c r="B29" s="8"/>
       <c r="C29" s="3"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="2"/>
+    <row r="30" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A30" s="27"/>
       <c r="B30" s="1"/>
       <c r="C30" s="9"/>
       <c r="D30" s="5"/>
       <c r="E30" s="5"/>
       <c r="F30" s="5"/>
+    </row>
+    <row r="31" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B31" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D31" t="s">
+        <v>67</v>
+      </c>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+    </row>
+    <row r="33" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B33" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E35" s="10"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="B36" t="s">
+        <v>69</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D36" t="s">
+        <v>70</v>
+      </c>
+      <c r="E36" s="10"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="B37" t="s">
+        <v>71</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D37" t="s">
+        <v>72</v>
+      </c>
+      <c r="E37" s="10"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="B38" t="s">
+        <v>73</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D38" t="s">
+        <v>74</v>
+      </c>
+      <c r="E38" s="10"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="B39" t="s">
+        <v>75</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D39" t="s">
+        <v>76</v>
+      </c>
+      <c r="E39" s="10"/>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+    </row>
+    <row r="41" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A41" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A42" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="B42" s="11" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="B43" t="s">
+        <v>79</v>
+      </c>
+      <c r="C43" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="B44" t="s">
+        <v>80</v>
+      </c>
+      <c r="C44" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="D44" t="s">
+        <v>81</v>
+      </c>
+      <c r="E44" t="s">
+        <v>82</v>
+      </c>
+      <c r="F44" t="s">
+        <v>83</v>
+      </c>
+      <c r="G44" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="19"/>
+      <c r="C45" s="14"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="13"/>
+      <c r="B46" s="12"/>
+      <c r="C46" s="14"/>
+      <c r="E46" s="12"/>
+      <c r="F46" s="12"/>
+    </row>
+    <row r="47" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A47" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="C47" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="D47" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A49" s="4"/>
+      <c r="B49" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A50" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="E50" s="7" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B51" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="C51" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="D51" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="E51" s="10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B52" s="21"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B53" s="21"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="B54" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="C54" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="D54" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="E54" s="23" t="s">
+        <v>96</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1078,18 +1540,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1316,6 +1778,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12EAFE4B-1F2D-4650-ACDE-3590E8305080}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{137977AE-5CF3-42F0-AD7C-49AF06AF507F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -1328,14 +1798,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="e1c8ebbc-f196-4c28-98e9-1900bd408e79"/>
     <ds:schemaRef ds:uri="bc8b8595-9fa1-49bc-a016-2621e7bde64e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12EAFE4B-1F2D-4650-ACDE-3590E8305080}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>